<commit_message>
changes for the paper
</commit_message>
<xml_diff>
--- a/data/crops/lu_c_factor_reducedtillage.xlsx
+++ b/data/crops/lu_c_factor_reducedtillage.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://worldwildlifefund-my.sharepoint.com/personal/cristobal_loyola_wwfus_org/Documents/Documents/203. Python projects/SBTN_Test/data/crops/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="82" documentId="8_{DE03094A-62C0-4937-830E-90DB4B2587C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{27DF468F-955A-40E3-B34F-D91DFFA9892B}"/>
+  <xr:revisionPtr revIDLastSave="86" documentId="8_{DE03094A-62C0-4937-830E-90DB4B2587C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2A6D869F-5FC4-4115-A285-1B9618839F49}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{AD288E80-6FC1-4BDD-A593-FC9351635447}"/>
   </bookViews>
@@ -419,12 +419,14 @@
       <sheetName val="Sheet1"/>
       <sheetName val="Crop_Classification"/>
       <sheetName val="C_Crops"/>
+      <sheetName val="lu_c_factor_inventory"/>
     </sheetNames>
     <sheetDataSet>
       <sheetData sheetId="0"/>
       <sheetData sheetId="1"/>
       <sheetData sheetId="2"/>
       <sheetData sheetId="3"/>
+      <sheetData sheetId="4" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -747,7 +749,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3D563D1-830A-486E-AE30-CC87FDA7651F}">
-  <dimension ref="A1:O27"/>
+  <dimension ref="A1:R27"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="49.453125" bestFit="1" customWidth="1"/>
@@ -759,7 +761,7 @@
     <col min="10" max="10" width="26.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -806,7 +808,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
         <v>13</v>
       </c>
@@ -855,7 +857,7 @@
         <v>6.1600000000000002E-2</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A3" s="7" t="s">
         <v>21</v>
       </c>
@@ -903,8 +905,16 @@
         <f t="shared" ref="O3:O27" si="1">+N3*M3*L3</f>
         <v>6.9999999999999993E-2</v>
       </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="Q3">
+        <f>+N3</f>
+        <v>0.35</v>
+      </c>
+      <c r="R3">
+        <f>+N4*M4</f>
+        <v>0.308</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
         <v>38</v>
       </c>
@@ -952,8 +962,16 @@
         <f t="shared" si="1"/>
         <v>6.1600000000000002E-2</v>
       </c>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="Q4">
+        <f>1-M2</f>
+        <v>0.12</v>
+      </c>
+      <c r="R4">
+        <f>1-R3</f>
+        <v>0.69199999999999995</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A5" s="7" t="s">
         <v>40</v>
       </c>
@@ -1002,7 +1020,7 @@
         <v>6.9999999999999993E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
         <v>23</v>
       </c>
@@ -1051,7 +1069,7 @@
         <v>0.11704000000000001</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A7" s="7" t="s">
         <v>25</v>
       </c>
@@ -1100,7 +1118,7 @@
         <v>0.13299999999999998</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A8" s="4" t="s">
         <v>41</v>
       </c>
@@ -1149,7 +1167,7 @@
         <v>0.11704000000000001</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A9" s="7" t="s">
         <v>42</v>
       </c>
@@ -1198,7 +1216,7 @@
         <v>0.13299999999999998</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A10" s="4" t="s">
         <v>26</v>
       </c>
@@ -1247,7 +1265,7 @@
         <v>7.6999999999999999E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A11" s="7" t="s">
         <v>29</v>
       </c>
@@ -1296,7 +1314,7 @@
         <v>8.7499999999999994E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A12" s="4" t="s">
         <v>43</v>
       </c>
@@ -1345,7 +1363,7 @@
         <v>7.6999999999999999E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A13" s="7" t="s">
         <v>44</v>
       </c>
@@ -1394,7 +1412,7 @@
         <v>8.7499999999999994E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A14" s="4" t="s">
         <v>30</v>
       </c>
@@ -1443,7 +1461,7 @@
         <v>3.0800000000000001E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A15" s="7" t="s">
         <v>34</v>
       </c>
@@ -1492,7 +1510,7 @@
         <v>3.4999999999999996E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A16" s="4" t="s">
         <v>45</v>
       </c>

</xml_diff>

<commit_message>
New threshold notebook. Changes to documentation to align with paper
</commit_message>
<xml_diff>
--- a/data/crops/lu_c_factor_reducedtillage.xlsx
+++ b/data/crops/lu_c_factor_reducedtillage.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://worldwildlifefund-my.sharepoint.com/personal/cristobal_loyola_wwfus_org/Documents/Documents/203. Python projects/SBTN_Test/data/crops/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="86" documentId="8_{DE03094A-62C0-4937-830E-90DB4B2587C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2A6D869F-5FC4-4115-A285-1B9618839F49}"/>
+  <xr:revisionPtr revIDLastSave="87" documentId="8_{DE03094A-62C0-4937-830E-90DB4B2587C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B8F45275-9D2B-49CD-B7E4-0579DDDD1CA3}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{AD288E80-6FC1-4BDD-A593-FC9351635447}"/>
   </bookViews>
@@ -749,7 +749,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3D563D1-830A-486E-AE30-CC87FDA7651F}">
-  <dimension ref="A1:R27"/>
+  <dimension ref="A1:O27"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="49.453125" bestFit="1" customWidth="1"/>
@@ -761,7 +761,7 @@
     <col min="10" max="10" width="26.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -808,7 +808,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
         <v>13</v>
       </c>
@@ -857,7 +857,7 @@
         <v>6.1600000000000002E-2</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A3" s="7" t="s">
         <v>21</v>
       </c>
@@ -905,16 +905,8 @@
         <f t="shared" ref="O3:O27" si="1">+N3*M3*L3</f>
         <v>6.9999999999999993E-2</v>
       </c>
-      <c r="Q3">
-        <f>+N3</f>
-        <v>0.35</v>
-      </c>
-      <c r="R3">
-        <f>+N4*M4</f>
-        <v>0.308</v>
-      </c>
-    </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.35">
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
         <v>38</v>
       </c>
@@ -962,16 +954,8 @@
         <f t="shared" si="1"/>
         <v>6.1600000000000002E-2</v>
       </c>
-      <c r="Q4">
-        <f>1-M2</f>
-        <v>0.12</v>
-      </c>
-      <c r="R4">
-        <f>1-R3</f>
-        <v>0.69199999999999995</v>
-      </c>
-    </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.35">
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A5" s="7" t="s">
         <v>40</v>
       </c>
@@ -1020,7 +1004,7 @@
         <v>6.9999999999999993E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
         <v>23</v>
       </c>
@@ -1069,7 +1053,7 @@
         <v>0.11704000000000001</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A7" s="7" t="s">
         <v>25</v>
       </c>
@@ -1118,7 +1102,7 @@
         <v>0.13299999999999998</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A8" s="4" t="s">
         <v>41</v>
       </c>
@@ -1167,7 +1151,7 @@
         <v>0.11704000000000001</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A9" s="7" t="s">
         <v>42</v>
       </c>
@@ -1216,7 +1200,7 @@
         <v>0.13299999999999998</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A10" s="4" t="s">
         <v>26</v>
       </c>
@@ -1265,7 +1249,7 @@
         <v>7.6999999999999999E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A11" s="7" t="s">
         <v>29</v>
       </c>
@@ -1314,7 +1298,7 @@
         <v>8.7499999999999994E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A12" s="4" t="s">
         <v>43</v>
       </c>
@@ -1363,7 +1347,7 @@
         <v>7.6999999999999999E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A13" s="7" t="s">
         <v>44</v>
       </c>
@@ -1412,7 +1396,7 @@
         <v>8.7499999999999994E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A14" s="4" t="s">
         <v>30</v>
       </c>
@@ -1461,7 +1445,7 @@
         <v>3.0800000000000001E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A15" s="7" t="s">
         <v>34</v>
       </c>
@@ -1510,7 +1494,7 @@
         <v>3.4999999999999996E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A16" s="4" t="s">
         <v>45</v>
       </c>

</xml_diff>